<commit_message>
Budget prévisionnel : cotisations réelles (babies, enfants, ados/adultes)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K99JAtbswA45kYPHTiReCE
</commit_message>
<xml_diff>
--- a/dojo/subvention/Budget_previsionnel_2026-2027.xlsx
+++ b/dojo/subvention/Budget_previsionnel_2026-2027.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="97">
   <si>
     <t xml:space="preserve">FIGHTER ACADEMY KARATE – SHIDOKAN RÉUNION</t>
   </si>
@@ -257,7 +257,13 @@
     <t xml:space="preserve">Adhérents</t>
   </si>
   <si>
-    <t xml:space="preserve">Nombre d'adhérents enfants (5-11 ans)</t>
+    <t xml:space="preserve">Nombre d'adhérents babies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cotisation annuelle baby</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nombre d'adhérents enfants</t>
   </si>
   <si>
     <t xml:space="preserve">Cotisation annuelle enfant</t>
@@ -1014,11 +1020,11 @@
         <v>16</v>
       </c>
       <c r="C12" s="10" t="n">
-        <f aca="false">Hypothèses!$B$14</f>
+        <f aca="false">Hypothèses!$B$16</f>
         <v>500</v>
       </c>
       <c r="D12" s="10" t="n">
-        <f aca="false">Hypothèses!$B$14</f>
+        <f aca="false">Hypothèses!$B$16</f>
         <v>500</v>
       </c>
     </row>
@@ -1030,11 +1036,11 @@
         <v>18</v>
       </c>
       <c r="C13" s="10" t="n">
-        <f aca="false">Hypothèses!$B$19</f>
+        <f aca="false">Hypothèses!$B$21</f>
         <v>300</v>
       </c>
       <c r="D13" s="10" t="n">
-        <f aca="false">Hypothèses!$B$19</f>
+        <f aca="false">Hypothèses!$B$21</f>
         <v>300</v>
       </c>
     </row>
@@ -1054,11 +1060,11 @@
         <v>21</v>
       </c>
       <c r="C15" s="10" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
+        <f aca="false">Hypothèses!$B$14</f>
         <v>400</v>
       </c>
       <c r="D15" s="10" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
+        <f aca="false">Hypothèses!$B$14</f>
         <v>400</v>
       </c>
     </row>
@@ -1120,11 +1126,11 @@
         <v>30</v>
       </c>
       <c r="C20" s="10" t="n">
-        <f aca="false">Hypothèses!$B$13</f>
+        <f aca="false">Hypothèses!$B$15</f>
         <v>2000</v>
       </c>
       <c r="D20" s="10" t="n">
-        <f aca="false">Hypothèses!$B$13</f>
+        <f aca="false">Hypothèses!$B$15</f>
         <v>2000</v>
       </c>
     </row>
@@ -1136,11 +1142,11 @@
         <v>31</v>
       </c>
       <c r="C21" s="10" t="n">
-        <f aca="false">Hypothèses!$B$15</f>
+        <f aca="false">Hypothèses!$B$17</f>
         <v>600</v>
       </c>
       <c r="D21" s="10" t="n">
-        <f aca="false">Hypothèses!$B$15</f>
+        <f aca="false">Hypothèses!$B$17</f>
         <v>600</v>
       </c>
     </row>
@@ -1152,11 +1158,11 @@
         <v>33</v>
       </c>
       <c r="C22" s="10" t="n">
-        <f aca="false">Hypothèses!$B$16</f>
+        <f aca="false">Hypothèses!$B$18</f>
         <v>300</v>
       </c>
       <c r="D22" s="10" t="n">
-        <f aca="false">Hypothèses!$B$16</f>
+        <f aca="false">Hypothèses!$B$18</f>
         <v>300</v>
       </c>
     </row>
@@ -1176,12 +1182,12 @@
         <v>36</v>
       </c>
       <c r="C24" s="10" t="n">
-        <f aca="false">(Hypothèses!$B$5+Hypothèses!$B$7)*Hypothèses!$B$10</f>
-        <v>1280</v>
+        <f aca="false">(Hypothèses!$B$5+Hypothèses!$B$7+Hypothèses!$B$9)*Hypothèses!$B$12</f>
+        <v>2520</v>
       </c>
       <c r="D24" s="10" t="n">
-        <f aca="false">(Hypothèses!$B$5+Hypothèses!$B$7)*Hypothèses!$B$10</f>
-        <v>1280</v>
+        <f aca="false">(Hypothèses!$B$5+Hypothèses!$B$7+Hypothèses!$B$9)*Hypothèses!$B$12</f>
+        <v>2520</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1192,11 +1198,11 @@
         <v>37</v>
       </c>
       <c r="C25" s="10" t="n">
-        <f aca="false">Hypothèses!$B$11</f>
+        <f aca="false">Hypothèses!$B$13</f>
         <v>150</v>
       </c>
       <c r="D25" s="10" t="n">
-        <f aca="false">Hypothèses!$B$11</f>
+        <f aca="false">Hypothèses!$B$13</f>
         <v>150</v>
       </c>
     </row>
@@ -1221,11 +1227,11 @@
       </c>
       <c r="C27" s="13" t="n">
         <f aca="false">SUM(C7:C26)</f>
-        <v>10530</v>
+        <v>11770</v>
       </c>
       <c r="D27" s="13" t="n">
         <f aca="false">SUM(D7:D26)</f>
-        <v>15530</v>
+        <v>16770</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1249,11 +1255,11 @@
         <v>44</v>
       </c>
       <c r="C31" s="10" t="n">
-        <f aca="false">Hypothèses!$B$18</f>
+        <f aca="false">Hypothèses!$B$20</f>
         <v>900</v>
       </c>
       <c r="D31" s="10" t="n">
-        <f aca="false">Hypothèses!$B$18</f>
+        <f aca="false">Hypothèses!$B$20</f>
         <v>900</v>
       </c>
     </row>
@@ -1337,12 +1343,12 @@
         <v>53</v>
       </c>
       <c r="C38" s="10" t="n">
-        <f aca="false">Hypothèses!$B$5*Hypothèses!$B$6+Hypothèses!$B$7*Hypothèses!$B$8</f>
-        <v>4200</v>
+        <f aca="false">Hypothèses!$B$5*Hypothèses!$B$6+Hypothèses!$B$7*Hypothèses!$B$8+Hypothèses!$B$9*Hypothèses!$B$10</f>
+        <v>17957</v>
       </c>
       <c r="D38" s="10" t="n">
-        <f aca="false">Hypothèses!$B$5*Hypothèses!$B$6+Hypothèses!$B$7*Hypothèses!$B$8</f>
-        <v>4200</v>
+        <f aca="false">Hypothèses!$B$5*Hypothèses!$B$6+Hypothèses!$B$7*Hypothèses!$B$8+Hypothèses!$B$9*Hypothèses!$B$10</f>
+        <v>17957</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1353,11 +1359,11 @@
         <v>55</v>
       </c>
       <c r="C39" s="10" t="n">
-        <f aca="false">Hypothèses!$B$20</f>
+        <f aca="false">Hypothèses!$B$22</f>
         <v>500</v>
       </c>
       <c r="D39" s="10" t="n">
-        <f aca="false">Hypothèses!$B$20</f>
+        <f aca="false">Hypothèses!$B$22</f>
         <v>500</v>
       </c>
     </row>
@@ -1368,11 +1374,11 @@
       </c>
       <c r="C40" s="15" t="n">
         <f aca="false">C27-SUM(C30:C39)</f>
-        <v>-70</v>
+        <v>-12587</v>
       </c>
       <c r="D40" s="15" t="n">
         <f aca="false">D27-SUM(D30:D39)</f>
-        <v>-70</v>
+        <v>-12587</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1382,11 +1388,11 @@
       </c>
       <c r="C41" s="13" t="n">
         <f aca="false">SUM(C30:C40)</f>
-        <v>10530</v>
+        <v>11770</v>
       </c>
       <c r="D41" s="13" t="n">
         <f aca="false">SUM(D30:D40)</f>
-        <v>15530</v>
+        <v>16770</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1410,11 +1416,11 @@
         <v>61</v>
       </c>
       <c r="C45" s="10" t="n">
-        <f aca="false">Hypothèses!$B$22*Hypothèses!$B$23</f>
+        <f aca="false">Hypothèses!$B$24*Hypothèses!$B$25</f>
         <v>4320</v>
       </c>
       <c r="D45" s="10" t="n">
-        <f aca="false">Hypothèses!$B$22*Hypothèses!$B$23</f>
+        <f aca="false">Hypothèses!$B$24*Hypothèses!$B$25</f>
         <v>4320</v>
       </c>
     </row>
@@ -1426,11 +1432,11 @@
         <v>63</v>
       </c>
       <c r="C46" s="10" t="n">
-        <f aca="false">Hypothèses!$B$24*Hypothèses!$B$25</f>
+        <f aca="false">Hypothèses!$B$26*Hypothèses!$B$27</f>
         <v>7800</v>
       </c>
       <c r="D46" s="10" t="n">
-        <f aca="false">Hypothèses!$B$24*Hypothèses!$B$25</f>
+        <f aca="false">Hypothèses!$B$26*Hypothèses!$B$27</f>
         <v>7800</v>
       </c>
     </row>
@@ -1464,11 +1470,11 @@
         <v>67</v>
       </c>
       <c r="C49" s="10" t="n">
-        <f aca="false">Hypothèses!$B$22*Hypothèses!$B$23</f>
+        <f aca="false">Hypothèses!$B$24*Hypothèses!$B$25</f>
         <v>4320</v>
       </c>
       <c r="D49" s="10" t="n">
-        <f aca="false">Hypothèses!$B$22*Hypothèses!$B$23</f>
+        <f aca="false">Hypothèses!$B$24*Hypothèses!$B$25</f>
         <v>4320</v>
       </c>
     </row>
@@ -1480,11 +1486,11 @@
         <v>69</v>
       </c>
       <c r="C50" s="10" t="n">
-        <f aca="false">Hypothèses!$B$24*Hypothèses!$B$25</f>
+        <f aca="false">Hypothèses!$B$26*Hypothèses!$B$27</f>
         <v>7800</v>
       </c>
       <c r="D50" s="10" t="n">
-        <f aca="false">Hypothèses!$B$24*Hypothèses!$B$25</f>
+        <f aca="false">Hypothèses!$B$26*Hypothèses!$B$27</f>
         <v>7800</v>
       </c>
     </row>
@@ -1521,11 +1527,11 @@
       </c>
       <c r="C54" s="21" t="n">
         <f aca="false">C33/C41</f>
-        <v>0.474833808167142</v>
+        <v>0.424808836023789</v>
       </c>
       <c r="D54" s="21" t="n">
         <f aca="false">D33/D41</f>
-        <v>0.643915003219575</v>
+        <v>0.596302921884317</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1554,7 +1560,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="62"/>
@@ -1582,7 +1588,7 @@
         <v>78</v>
       </c>
       <c r="B5" s="27" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1590,7 +1596,7 @@
         <v>79</v>
       </c>
       <c r="B6" s="28" t="n">
-        <v>120</v>
+        <v>239</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1598,7 +1604,7 @@
         <v>80</v>
       </c>
       <c r="B7" s="27" t="n">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1606,129 +1612,129 @@
         <v>81</v>
       </c>
       <c r="B8" s="28" t="n">
-        <v>150</v>
+        <v>259</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="25" t="s">
+      <c r="A9" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="B9" s="26"/>
+      <c r="B9" s="27" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
         <v>83</v>
       </c>
       <c r="B10" s="28" t="n">
-        <v>40</v>
+        <v>339</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="B11" s="28" t="n">
-        <v>150</v>
-      </c>
+      <c r="A11" s="25" t="s">
+        <v>84</v>
+      </c>
+      <c r="B11" s="26"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>21</v>
+        <v>85</v>
       </c>
       <c r="B12" s="28" t="n">
-        <v>400</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>84</v>
+        <v>37</v>
       </c>
       <c r="B13" s="28" t="n">
-        <v>2000</v>
+        <v>150</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B14" s="28" t="n">
-        <v>500</v>
+        <v>400</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B15" s="28" t="n">
-        <v>600</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="B16" s="28" t="n">
-        <v>300</v>
+        <v>500</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="B17" s="26"/>
+      <c r="A17" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="B17" s="28" t="n">
+        <v>600</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>87</v>
+        <v>33</v>
       </c>
       <c r="B18" s="28" t="n">
-        <v>900</v>
+        <v>300</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="8" t="s">
+      <c r="A19" s="25" t="s">
         <v>88</v>
       </c>
-      <c r="B19" s="28" t="n">
-        <v>300</v>
-      </c>
+      <c r="B19" s="26"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
         <v>89</v>
       </c>
       <c r="B20" s="28" t="n">
-        <v>500</v>
+        <v>900</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="25" t="s">
+      <c r="A21" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="B21" s="26"/>
+      <c r="B21" s="28" t="n">
+        <v>300</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="B22" s="27" t="n">
-        <v>216</v>
+      <c r="B22" s="28" t="n">
+        <v>500</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="8" t="s">
+      <c r="A23" s="25" t="s">
         <v>92</v>
       </c>
-      <c r="B23" s="28" t="n">
-        <v>20</v>
-      </c>
+      <c r="B23" s="26"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
         <v>93</v>
       </c>
       <c r="B24" s="27" t="n">
-        <v>650</v>
+        <v>216</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1736,6 +1742,22 @@
         <v>94</v>
       </c>
       <c r="B25" s="28" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="B26" s="27" t="n">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="B27" s="28" t="n">
         <v>12</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Budget prévisionnel : 63 adhérents, licence 39 €, affiliation Shidokan 21 €, matériel 1 200 €, encadrants bénévoles
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K99JAtbswA45kYPHTiReCE
</commit_message>
<xml_diff>
--- a/dojo/subvention/Budget_previsionnel_2026-2027.xlsx
+++ b/dojo/subvention/Budget_previsionnel_2026-2027.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="98">
   <si>
     <t xml:space="preserve">FIGHTER ACADEMY KARATE – SHIDOKAN RÉUNION</t>
   </si>
@@ -134,7 +134,7 @@
     <t xml:space="preserve">Licences fédérales</t>
   </si>
   <si>
-    <t xml:space="preserve">Affiliation du club à la fédération</t>
+    <t xml:space="preserve">Affiliation Shidokan (par adhérent)</t>
   </si>
   <si>
     <t xml:space="preserve">6588</t>
@@ -279,6 +279,9 @@
   </si>
   <si>
     <t xml:space="preserve">Prix de la licence fédérale par adhérent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Affiliation Shidokan par adhérent</t>
   </si>
   <si>
     <t xml:space="preserve">Déplacements en compétition (transport, engagements)</t>
@@ -1021,11 +1024,11 @@
       </c>
       <c r="C12" s="10" t="n">
         <f aca="false">Hypothèses!$B$16</f>
-        <v>500</v>
+        <v>1200</v>
       </c>
       <c r="D12" s="10" t="n">
         <f aca="false">Hypothèses!$B$16</f>
-        <v>500</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1127,11 +1130,11 @@
       </c>
       <c r="C20" s="10" t="n">
         <f aca="false">Hypothèses!$B$15</f>
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="D20" s="10" t="n">
         <f aca="false">Hypothèses!$B$15</f>
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1143,11 +1146,11 @@
       </c>
       <c r="C21" s="10" t="n">
         <f aca="false">Hypothèses!$B$17</f>
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="D21" s="10" t="n">
         <f aca="false">Hypothèses!$B$17</f>
-        <v>600</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1183,11 +1186,11 @@
       </c>
       <c r="C24" s="10" t="n">
         <f aca="false">(Hypothèses!$B$5+Hypothèses!$B$7+Hypothèses!$B$9)*Hypothèses!$B$12</f>
-        <v>2520</v>
+        <v>2457</v>
       </c>
       <c r="D24" s="10" t="n">
         <f aca="false">(Hypothèses!$B$5+Hypothèses!$B$7+Hypothèses!$B$9)*Hypothèses!$B$12</f>
-        <v>2520</v>
+        <v>2457</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1198,12 +1201,12 @@
         <v>37</v>
       </c>
       <c r="C25" s="10" t="n">
-        <f aca="false">Hypothèses!$B$13</f>
-        <v>150</v>
+        <f aca="false">(Hypothèses!$B$5+Hypothèses!$B$7+Hypothèses!$B$9)*Hypothèses!$B$13</f>
+        <v>1323</v>
       </c>
       <c r="D25" s="10" t="n">
-        <f aca="false">Hypothèses!$B$13</f>
-        <v>150</v>
+        <f aca="false">(Hypothèses!$B$5+Hypothèses!$B$7+Hypothèses!$B$9)*Hypothèses!$B$13</f>
+        <v>1323</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1227,11 +1230,11 @@
       </c>
       <c r="C27" s="13" t="n">
         <f aca="false">SUM(C7:C26)</f>
-        <v>11770</v>
+        <v>10980</v>
       </c>
       <c r="D27" s="13" t="n">
         <f aca="false">SUM(D7:D26)</f>
-        <v>16770</v>
+        <v>15980</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1374,11 +1377,11 @@
       </c>
       <c r="C40" s="15" t="n">
         <f aca="false">C27-SUM(C30:C39)</f>
-        <v>-12587</v>
+        <v>-13377</v>
       </c>
       <c r="D40" s="15" t="n">
         <f aca="false">D27-SUM(D30:D39)</f>
-        <v>-12587</v>
+        <v>-13377</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1388,11 +1391,11 @@
       </c>
       <c r="C41" s="13" t="n">
         <f aca="false">SUM(C30:C40)</f>
-        <v>11770</v>
+        <v>10980</v>
       </c>
       <c r="D41" s="13" t="n">
         <f aca="false">SUM(D30:D40)</f>
-        <v>16770</v>
+        <v>15980</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1527,11 +1530,11 @@
       </c>
       <c r="C54" s="21" t="n">
         <f aca="false">C33/C41</f>
-        <v>0.424808836023789</v>
+        <v>0.455373406193078</v>
       </c>
       <c r="D54" s="21" t="n">
         <f aca="false">D33/D41</f>
-        <v>0.596302921884317</v>
+        <v>0.625782227784731</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1642,15 +1645,15 @@
         <v>85</v>
       </c>
       <c r="B12" s="28" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>37</v>
+        <v>86</v>
       </c>
       <c r="B13" s="28" t="n">
-        <v>150</v>
+        <v>21</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1663,10 +1666,10 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B15" s="28" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1674,15 +1677,15 @@
         <v>16</v>
       </c>
       <c r="B16" s="28" t="n">
-        <v>500</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B17" s="28" t="n">
-        <v>600</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1695,13 +1698,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="25" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B19" s="26"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B20" s="28" t="n">
         <v>900</v>
@@ -1709,7 +1712,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B21" s="28" t="n">
         <v>300</v>
@@ -1717,7 +1720,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B22" s="28" t="n">
         <v>500</v>
@@ -1725,13 +1728,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="25" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B23" s="26"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B24" s="27" t="n">
         <v>216</v>
@@ -1739,7 +1742,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B25" s="28" t="n">
         <v>20</v>
@@ -1747,7 +1750,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="8" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B26" s="27" t="n">
         <v>650</v>
@@ -1755,7 +1758,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="8" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B27" s="28" t="n">
         <v>12</v>

</xml_diff>